<commit_message>
espectros de ESPARTACO 2
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,20 +451,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Velocidad [km/s]</t>
+          <t>Velocidad obs. [km/s]</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Velocidad heliocéntrica [km/s]</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Profundidad / Altura</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>FWHM [Å]</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>EW [Å]</t>
         </is>
@@ -488,15 +493,18 @@
         <v>6.4e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>19.0999</v>
+        <v>19.1</v>
       </c>
       <c r="F2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G2" t="n">
         <v>0.4944</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.927</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.5872000000000001</v>
       </c>
     </row>
@@ -521,12 +529,15 @@
         <v>21.86</v>
       </c>
       <c r="F3" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.5265</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.883</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.5611</v>
       </c>
     </row>
@@ -551,12 +562,15 @@
         <v>27.47</v>
       </c>
       <c r="F4" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.4879</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.926</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.5868</v>
       </c>
     </row>
@@ -581,12 +595,15 @@
         <v>28.69</v>
       </c>
       <c r="F5" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.5288</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.968</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.6183</v>
       </c>
     </row>
@@ -611,12 +628,15 @@
         <v>28.76</v>
       </c>
       <c r="F6" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.4869</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>1.008</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>0.6425999999999999</v>
       </c>
     </row>
@@ -641,12 +661,15 @@
         <v>27.73</v>
       </c>
       <c r="F7" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.5024999999999999</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>1.002</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>0.639</v>
       </c>
     </row>
@@ -671,12 +694,15 @@
         <v>27.14</v>
       </c>
       <c r="F8" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="G8" t="n">
         <v>0.4998</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>1.041</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>0.6685</v>
       </c>
     </row>
@@ -701,12 +727,15 @@
         <v>26.71</v>
       </c>
       <c r="F9" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G9" t="n">
         <v>0.5061</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>1.025</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>0.6525</v>
       </c>
     </row>
@@ -731,12 +760,15 @@
         <v>22.64</v>
       </c>
       <c r="F10" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="G10" t="n">
         <v>0.5544</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>1.053</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>0.6811</v>
       </c>
     </row>
@@ -761,12 +793,15 @@
         <v>20.25</v>
       </c>
       <c r="F11" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="G11" t="n">
         <v>0.5538</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>1.043</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>0.6707</v>
       </c>
     </row>
@@ -791,12 +826,15 @@
         <v>19.8</v>
       </c>
       <c r="F12" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="G12" t="n">
         <v>0.5034999999999999</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>1.025</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>0.6525</v>
       </c>
     </row>
@@ -821,12 +859,15 @@
         <v>17.87</v>
       </c>
       <c r="F13" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="G13" t="n">
         <v>0.5184</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>1.04</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>0.6683</v>
       </c>
     </row>
@@ -851,12 +892,15 @@
         <v>18.07</v>
       </c>
       <c r="F14" t="n">
+        <v>-5.06</v>
+      </c>
+      <c r="G14" t="n">
         <v>0.4884</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>1.025</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>0.6531</v>
       </c>
     </row>
@@ -881,12 +925,15 @@
         <v>18.19</v>
       </c>
       <c r="F15" t="n">
+        <v>-5.74</v>
+      </c>
+      <c r="G15" t="n">
         <v>0.5004</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>1.027</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>0.6543</v>
       </c>
     </row>
@@ -911,12 +958,15 @@
         <v>20.64</v>
       </c>
       <c r="F16" t="n">
+        <v>-5.86</v>
+      </c>
+      <c r="G16" t="n">
         <v>0.4954</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>1.025</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>0.6525</v>
       </c>
     </row>
@@ -941,12 +991,15 @@
         <v>21.77</v>
       </c>
       <c r="F17" t="n">
+        <v>-5.88</v>
+      </c>
+      <c r="G17" t="n">
         <v>0.4977</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>1.041</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>0.6685</v>
       </c>
     </row>
@@ -971,12 +1024,15 @@
         <v>21.59</v>
       </c>
       <c r="F18" t="n">
+        <v>-6.23</v>
+      </c>
+      <c r="G18" t="n">
         <v>0.4917</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>1.052</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>0.6801</v>
       </c>
     </row>
@@ -1001,12 +1057,15 @@
         <v>25.15</v>
       </c>
       <c r="F19" t="n">
+        <v>-4.34</v>
+      </c>
+      <c r="G19" t="n">
         <v>0.5489000000000001</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>1.07</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>0.6982</v>
       </c>
     </row>
@@ -1031,13 +1090,115 @@
         <v>24.07</v>
       </c>
       <c r="F20" t="n">
+        <v>-5.44</v>
+      </c>
+      <c r="G20" t="n">
         <v>0.5484</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>1.126</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>0.7531</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Septiembre 14-2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6563.914</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7.9e-05</v>
+      </c>
+      <c r="E21" t="n">
+        <v>23.63</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.5512</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.7586000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Septiembre 21-2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6563.894</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7.6e-05</v>
+      </c>
+      <c r="E22" t="n">
+        <v>22.71</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.5586</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.121</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.7483</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Septiembre 29-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6563.856</v>
+      </c>
+      <c r="D23" t="n">
+        <v>6.999999999999999e-05</v>
+      </c>
+      <c r="E23" t="n">
+        <v>20.95</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-5.63</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.5543</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.7606000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
datos 2024 y 2026 arreglados
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
@@ -487,25 +487,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6563.815</v>
+        <v>6563.814</v>
       </c>
       <c r="D2" t="n">
         <v>6.4e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>19.1</v>
+        <v>19.04</v>
       </c>
       <c r="F2" t="n">
-        <v>0.45</v>
+        <v>0.39</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4944</v>
+        <v>0.4981</v>
       </c>
       <c r="H2" t="n">
-        <v>0.927</v>
+        <v>0.904</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5872000000000001</v>
+        <v>0.5735</v>
       </c>
     </row>
     <row r="3">
@@ -538,7 +538,7 @@
         <v>0.883</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5611</v>
+        <v>0.5610000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -565,7 +565,7 @@
         <v>-0.87</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4879</v>
+        <v>0.4888</v>
       </c>
       <c r="H4" t="n">
         <v>0.926</v>
@@ -598,13 +598,13 @@
         <v>-0.66</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5288</v>
+        <v>0.5301</v>
       </c>
       <c r="H5" t="n">
-        <v>0.968</v>
+        <v>0.958</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6183</v>
+        <v>0.6122</v>
       </c>
     </row>
     <row r="6">
@@ -631,13 +631,13 @@
         <v>-0.8100000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4869</v>
+        <v>0.4903</v>
       </c>
       <c r="H6" t="n">
-        <v>1.008</v>
+        <v>0.973</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6425999999999999</v>
+        <v>0.6217</v>
       </c>
     </row>
     <row r="7">
@@ -667,10 +667,10 @@
         <v>0.5024999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>1.002</v>
+        <v>1.003</v>
       </c>
       <c r="I7" t="n">
-        <v>0.639</v>
+        <v>0.6393</v>
       </c>
     </row>
     <row r="8">
@@ -763,13 +763,13 @@
         <v>-0.47</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5544</v>
+        <v>0.5558</v>
       </c>
       <c r="H10" t="n">
-        <v>1.053</v>
+        <v>1.056</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6811</v>
+        <v>0.6843</v>
       </c>
     </row>
     <row r="11">
@@ -796,13 +796,13 @@
         <v>-0.8</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5538</v>
+        <v>0.555</v>
       </c>
       <c r="H11" t="n">
-        <v>1.043</v>
+        <v>1.05</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6707</v>
+        <v>0.6783</v>
       </c>
     </row>
     <row r="12">
@@ -829,7 +829,7 @@
         <v>-0.92</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5034999999999999</v>
+        <v>0.5037</v>
       </c>
       <c r="H12" t="n">
         <v>1.025</v>
@@ -862,13 +862,13 @@
         <v>-0.5600000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5184</v>
+        <v>0.5172</v>
       </c>
       <c r="H13" t="n">
-        <v>1.04</v>
+        <v>1.07</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6683</v>
+        <v>0.6977</v>
       </c>
     </row>
     <row r="14">
@@ -898,10 +898,10 @@
         <v>0.4884</v>
       </c>
       <c r="H14" t="n">
-        <v>1.025</v>
+        <v>1.026</v>
       </c>
       <c r="I14" t="n">
-        <v>0.6531</v>
+        <v>0.6538</v>
       </c>
     </row>
     <row r="15">
@@ -931,10 +931,10 @@
         <v>0.5004</v>
       </c>
       <c r="H15" t="n">
-        <v>1.027</v>
+        <v>1.025</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6543</v>
+        <v>0.6525</v>
       </c>
     </row>
     <row r="16">
@@ -961,7 +961,7 @@
         <v>-5.86</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4954</v>
+        <v>0.4953</v>
       </c>
       <c r="H16" t="n">
         <v>1.025</v>
@@ -994,7 +994,7 @@
         <v>-5.88</v>
       </c>
       <c r="G17" t="n">
-        <v>0.4977</v>
+        <v>0.4979</v>
       </c>
       <c r="H17" t="n">
         <v>1.041</v>
@@ -1027,13 +1027,13 @@
         <v>-6.23</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4917</v>
+        <v>0.4919</v>
       </c>
       <c r="H18" t="n">
-        <v>1.052</v>
+        <v>1.046</v>
       </c>
       <c r="I18" t="n">
-        <v>0.6801</v>
+        <v>0.6741</v>
       </c>
     </row>
     <row r="19">
@@ -1060,13 +1060,13 @@
         <v>-4.34</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.5496</v>
       </c>
       <c r="H19" t="n">
-        <v>1.07</v>
+        <v>1.068</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6982</v>
+        <v>0.6957</v>
       </c>
     </row>
     <row r="20">
@@ -1096,10 +1096,10 @@
         <v>0.5484</v>
       </c>
       <c r="H20" t="n">
-        <v>1.126</v>
+        <v>1.132</v>
       </c>
       <c r="I20" t="n">
-        <v>0.7531</v>
+        <v>0.7595</v>
       </c>
     </row>
     <row r="21">
@@ -1126,13 +1126,13 @@
         <v>-5.33</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5512</v>
+        <v>0.5528</v>
       </c>
       <c r="H21" t="n">
-        <v>1.131</v>
+        <v>1.149</v>
       </c>
       <c r="I21" t="n">
-        <v>0.7586000000000001</v>
+        <v>0.776</v>
       </c>
     </row>
     <row r="22">
@@ -1192,13 +1192,13 @@
         <v>-5.63</v>
       </c>
       <c r="G23" t="n">
-        <v>0.5543</v>
+        <v>0.5547</v>
       </c>
       <c r="H23" t="n">
-        <v>1.133</v>
+        <v>1.14</v>
       </c>
       <c r="I23" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.7673</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
parametros espectros 2025 y 2026
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados absorción cobalto 2024, 2025 y 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -898,7 +898,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Julio 24-2026</t>
+          <t>Agosto 19-2025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -907,21 +907,21 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6563.793</v>
+        <v>6563.989</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>6e-05</t>
+          <t>9e-05</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>18.07</v>
+        <v>27.05</v>
       </c>
       <c r="F14" t="n">
-        <v>-5.06</v>
+        <v>-1.75</v>
       </c>
       <c r="G14" t="n">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="H14" t="n">
         <v>1.03</v>
@@ -933,7 +933,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Julio 27-2026</t>
+          <t>Julio 24-2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -942,24 +942,24 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6563.795</v>
+        <v>6563.793</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.1e-05</t>
+          <t>6e-05</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>18.19</v>
+        <v>18.07</v>
       </c>
       <c r="F15" t="n">
-        <v>-5.74</v>
+        <v>-5.06</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="H15" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="I15" t="n">
         <v>0.65</v>
@@ -968,7 +968,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Agosto 06-2026</t>
+          <t>Julio 27-2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -977,18 +977,18 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6563.849</v>
+        <v>6563.795</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.9e-05</t>
+          <t>6.1e-05</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>20.64</v>
+        <v>18.19</v>
       </c>
       <c r="F16" t="n">
-        <v>-5.86</v>
+        <v>-5.74</v>
       </c>
       <c r="G16" t="n">
         <v>0.5</v>
@@ -1003,7 +1003,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Agosto 10-2026</t>
+          <t>Agosto 06-2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1012,33 +1012,33 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6563.874</v>
+        <v>6563.849</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>7.3e-05</t>
+          <t>6.9e-05</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>21.77</v>
+        <v>20.64</v>
       </c>
       <c r="F17" t="n">
-        <v>-5.88</v>
+        <v>-5.86</v>
       </c>
       <c r="G17" t="n">
         <v>0.5</v>
       </c>
       <c r="H17" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="I17" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Agosto 13-2026</t>
+          <t>Agosto 10-2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1047,24 +1047,24 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6563.87</v>
+        <v>6563.874</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.2e-05</t>
+          <t>7.3e-05</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>21.59</v>
+        <v>21.77</v>
       </c>
       <c r="F18" t="n">
-        <v>-6.23</v>
+        <v>-5.88</v>
       </c>
       <c r="G18" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="H18" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="I18" t="n">
         <v>0.67</v>
@@ -1073,7 +1073,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Agosto 28-2026</t>
+          <t>Agosto 13-2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1082,33 +1082,33 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6563.948</v>
+        <v>6563.87</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>8.4e-05</t>
+          <t>7.2e-05</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>25.15</v>
+        <v>21.59</v>
       </c>
       <c r="F19" t="n">
-        <v>-4.34</v>
+        <v>-6.23</v>
       </c>
       <c r="G19" t="n">
-        <v>0.55</v>
+        <v>0.49</v>
       </c>
       <c r="H19" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="I19" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Septiembre 07-2026</t>
+          <t>Agosto 28-2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1117,33 +1117,33 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6563.924</v>
+        <v>6563.948</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>8e-05</t>
+          <t>8.4e-05</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>24.07</v>
+        <v>25.15</v>
       </c>
       <c r="F20" t="n">
-        <v>-5.44</v>
+        <v>-4.34</v>
       </c>
       <c r="G20" t="n">
         <v>0.55</v>
       </c>
       <c r="H20" t="n">
-        <v>1.13</v>
+        <v>1.07</v>
       </c>
       <c r="I20" t="n">
-        <v>0.76</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Septiembre 14-2026</t>
+          <t>Septiembre 07-2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1152,33 +1152,33 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6563.914</v>
+        <v>6563.924</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7.9e-05</t>
+          <t>8e-05</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>23.63</v>
+        <v>24.07</v>
       </c>
       <c r="F21" t="n">
-        <v>-5.33</v>
+        <v>-5.44</v>
       </c>
       <c r="G21" t="n">
         <v>0.55</v>
       </c>
       <c r="H21" t="n">
-        <v>1.15</v>
+        <v>1.13</v>
       </c>
       <c r="I21" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Septiembre 21-2026</t>
+          <t>Septiembre 14-2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1187,62 +1187,132 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6563.894</v>
+        <v>6563.914</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>7.6e-05</t>
+          <t>7.9e-05</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>22.71</v>
+        <v>23.63</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.5</v>
+        <v>-5.33</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="H22" t="n">
-        <v>1.12</v>
+        <v>1.15</v>
       </c>
       <c r="I22" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Septiembre 21-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6563.894</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>7.6e-05</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>22.71</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Septiembre 29-2026</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Absorción Cobalto</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>6563.856</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>7e-05</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E24" t="n">
         <v>20.95</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F24" t="n">
         <v>-5.63</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G24" t="n">
         <v>0.55</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H24" t="n">
         <v>1.14</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I24" t="n">
         <v>0.77</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Octubre 16-2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>6563.711</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>4.8e-05</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>14.36</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-7.25</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>